<commit_message>
add dpGWP with fixed CO2
</commit_message>
<xml_diff>
--- a/dpLCIA/LCIA/premise_gwp/lcia_gwp2021_100a_w_bio_map_minorGHG_AR6_fair.xlsx
+++ b/dpLCIA/LCIA/premise_gwp/lcia_gwp2021_100a_w_bio_map_minorGHG_AR6_fair.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susierwu/dpLCA_main/dpLCIA/LCIA/premise_gwp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F26CA71-DB89-6D46-A4C7-A6FD149F7A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC709C23-2F7C-9C48-95DF-11195FE001B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="2080" windowWidth="24460" windowHeight="13500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2700" yWindow="1200" windowWidth="26100" windowHeight="15520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="premise_flows" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">premise_flows!$A$1:$C$256</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1123,7 +1123,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1132,7 +1132,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1192,16 +1191,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>105833</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>116417</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:rowOff>158751</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>800098</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>810682</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>55266</xdr:rowOff>
+      <xdr:rowOff>182267</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1223,7 +1222,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1862666" y="232833"/>
+          <a:off x="5069417" y="359834"/>
           <a:ext cx="3996265" cy="2838683"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6295,7 +6294,7 @@
       <c r="G123" s="2">
         <v>11200</v>
       </c>
-      <c r="H123" s="8" t="s">
+      <c r="H123" t="s">
         <v>193</v>
       </c>
     </row>
@@ -7871,91 +7870,91 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9685C091-66AB-2C4E-929B-EDC6397F5B69}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="32.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:5">
       <c r="A11" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:5">
       <c r="A13" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:5">
       <c r="A15" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
         <v>97</v>
       </c>
@@ -9789,7 +9788,7 @@
       <c r="G123" s="2">
         <v>11200</v>
       </c>
-      <c r="H123" s="8" t="s">
+      <c r="H123" t="s">
         <v>193</v>
       </c>
     </row>

</xml_diff>